<commit_message>
fix: simplify curse of dimensionality
</commit_message>
<xml_diff>
--- a/program.xlsx
+++ b/program.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\repos\teaching\AA2627-unibo-mldm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D22F050-EB1B-4DA9-B79B-05FE1EA1B4FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C6EB7B1-2977-4A54-8E96-AB4AE48CF762}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="72" yWindow="24" windowWidth="30168" windowHeight="14388" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2304" yWindow="2304" windowWidth="34560" windowHeight="18600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AA2627" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="54">
   <si>
     <t>When</t>
   </si>
@@ -86,18 +86,12 @@
     <t>Lab-Classification</t>
   </si>
   <si>
-    <t>05-NN</t>
-  </si>
-  <si>
     <t>Modeling</t>
   </si>
   <si>
     <t>Clustering</t>
   </si>
   <si>
-    <t>Ensemble?</t>
-  </si>
-  <si>
     <t>-</t>
   </si>
   <si>
@@ -201,6 +195,9 @@
   </si>
   <si>
     <t>Evaluation + 03-KNN</t>
+  </si>
+  <si>
+    <t>05-NN + Ensemble?</t>
   </si>
 </sst>
 </file>
@@ -666,7 +663,7 @@
         <v>9</v>
       </c>
       <c r="E2" s="19" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G2" s="7">
         <v>3</v>
@@ -691,7 +688,7 @@
         <v>11</v>
       </c>
       <c r="E3" s="19" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="G3" s="7">
         <v>2</v>
@@ -740,8 +737,8 @@
       <c r="D5" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="E5" t="s">
-        <v>54</v>
+      <c r="E5" s="19" t="s">
+        <v>52</v>
       </c>
       <c r="G5" s="7">
         <v>2</v>
@@ -793,7 +790,7 @@
         <v>11</v>
       </c>
       <c r="E7" s="15" t="s">
-        <v>16</v>
+        <v>53</v>
       </c>
       <c r="G7" s="7">
         <v>2</v>
@@ -819,7 +816,7 @@
         <v>9</v>
       </c>
       <c r="E8" s="15" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G8" s="7">
         <v>3</v>
@@ -845,10 +842,7 @@
         <v>11</v>
       </c>
       <c r="E9" t="s">
-        <v>18</v>
-      </c>
-      <c r="F9" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="G9" s="7">
         <v>2</v>
@@ -874,10 +868,10 @@
         <v>9</v>
       </c>
       <c r="E10" s="15" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="H10" s="16">
         <f>SUM($G$2:G10)/$G$20</f>
@@ -900,10 +894,10 @@
         <v>11</v>
       </c>
       <c r="E11" s="15" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="H11" s="16">
         <f>SUM($G$2:G11)/$G$20</f>
@@ -926,10 +920,10 @@
         <v>9</v>
       </c>
       <c r="E12" s="17" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="H12" s="16">
         <f>SUM($G$2:G12)/$G$20</f>
@@ -952,10 +946,10 @@
         <v>11</v>
       </c>
       <c r="E13" s="17" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="H13" s="16">
         <f>SUM($G$2:G13)/$G$20</f>
@@ -978,7 +972,7 @@
         <v>9</v>
       </c>
       <c r="E14" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G14" s="7">
         <v>3</v>
@@ -1004,7 +998,7 @@
         <v>11</v>
       </c>
       <c r="E15" s="15" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="G15" s="7">
         <v>2</v>
@@ -1030,7 +1024,7 @@
         <v>9</v>
       </c>
       <c r="E16" s="15" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="G16" s="7">
         <v>3</v>
@@ -1056,7 +1050,7 @@
         <v>11</v>
       </c>
       <c r="E17" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="G17" s="7">
         <v>2</v>
@@ -1071,7 +1065,7 @@
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="E19" s="9" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="G19" s="5">
         <f>SUM(G2:G17)</f>
@@ -1081,7 +1075,7 @@
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="E20" s="9" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="G20" s="1">
         <v>30</v>
@@ -1157,16 +1151,16 @@
         <v>3</v>
       </c>
       <c r="C2" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F2" t="s">
         <v>25</v>
-      </c>
-      <c r="D2" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="E2" t="s">
-        <v>26</v>
-      </c>
-      <c r="F2" t="s">
-        <v>27</v>
       </c>
       <c r="G2" s="7">
         <v>2</v>
@@ -1186,16 +1180,16 @@
         <v>3</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D3" s="8" t="s">
         <v>11</v>
       </c>
       <c r="E3" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="F3" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G3" s="7">
         <v>2</v>
@@ -1215,16 +1209,16 @@
         <v>3</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D4" s="8" t="s">
         <v>11</v>
       </c>
       <c r="E4" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F4" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="G4" s="7">
         <v>2</v>
@@ -1244,13 +1238,13 @@
         <v>3</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>9</v>
       </c>
       <c r="E5" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="G5" s="7">
         <v>2</v>
@@ -1270,13 +1264,13 @@
         <v>3</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D6" s="8" t="s">
         <v>11</v>
       </c>
       <c r="E6" s="15" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="G6" s="7">
         <v>2</v>
@@ -1296,16 +1290,16 @@
         <v>3</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D7" s="8" t="s">
         <v>11</v>
       </c>
       <c r="E7" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F7" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G7" s="7">
         <v>2</v>
@@ -1325,13 +1319,13 @@
         <v>3</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D8" s="8" t="s">
         <v>11</v>
       </c>
       <c r="E8" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="G8" s="7">
         <v>2</v>
@@ -1351,13 +1345,13 @@
         <v>3</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>9</v>
       </c>
       <c r="E9" s="15" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="G9" s="7">
         <v>2</v>
@@ -1377,13 +1371,13 @@
         <v>3</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>9</v>
       </c>
       <c r="E10" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="G10" s="7">
         <v>2</v>
@@ -1403,13 +1397,13 @@
         <v>3</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D11" s="8" t="s">
         <v>11</v>
       </c>
       <c r="E11" s="15" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="G11" s="7">
         <v>2</v>
@@ -1429,13 +1423,13 @@
         <v>3</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D12" s="5" t="s">
         <v>9</v>
       </c>
       <c r="E12" s="17" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G12" s="7">
         <v>2</v>
@@ -1455,13 +1449,13 @@
         <v>3</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>9</v>
       </c>
       <c r="E13" s="17" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G13" s="7">
         <v>2</v>
@@ -1481,11 +1475,11 @@
         <v>3</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D14" s="5"/>
       <c r="G14" s="7" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="H14" s="4">
         <f>SUM($G$2:G14)/$G$17</f>
@@ -1498,7 +1492,7 @@
       <c r="C15" s="10"/>
       <c r="D15" s="5"/>
       <c r="G15" s="5" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="H15" s="4">
         <f>SUM($G$2:G15)/$G$17</f>
@@ -1511,7 +1505,7 @@
       <c r="C16" s="13"/>
       <c r="D16" s="6"/>
       <c r="E16" s="9" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="G16" s="5">
         <f>SUM(G2:G14)</f>
@@ -1521,7 +1515,7 @@
     </row>
     <row r="17" spans="5:7" x14ac:dyDescent="0.3">
       <c r="E17" s="9" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="G17" s="1">
         <v>24</v>
@@ -1578,7 +1572,7 @@
         <v>4</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="G1" s="3" t="s">
         <v>6</v>
@@ -1597,16 +1591,16 @@
         <v>2</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D2" s="8" t="s">
         <v>11</v>
       </c>
       <c r="E2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="G2" s="7">
         <v>2</v>
@@ -1626,16 +1620,16 @@
         <v>2</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D3" s="8" t="s">
         <v>11</v>
       </c>
       <c r="E3" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="F3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="G3" s="7">
         <v>2</v>
@@ -1655,13 +1649,13 @@
         <v>2</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>9</v>
       </c>
       <c r="E4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="G4" s="7">
         <v>2</v>
@@ -1681,13 +1675,13 @@
         <v>2</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D5" s="8" t="s">
         <v>11</v>
       </c>
       <c r="E5" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="G5" s="7">
         <v>2</v>
@@ -1707,13 +1701,13 @@
         <v>2</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D6" s="8" t="s">
         <v>11</v>
       </c>
       <c r="E6" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="G6" s="7">
         <v>2</v>
@@ -1733,13 +1727,13 @@
         <v>2</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>9</v>
       </c>
       <c r="E7" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G7" s="7">
         <v>2</v>
@@ -1759,16 +1753,16 @@
         <v>2</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E8" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="H8" s="4">
         <f>SUM($G$2:G8)/$G$17</f>
@@ -1785,13 +1779,13 @@
         <v>2</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D9" s="8" t="s">
         <v>11</v>
       </c>
       <c r="E9" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="G9" s="7">
         <v>2</v>
@@ -1811,13 +1805,13 @@
         <v>2</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D10" s="8" t="s">
         <v>11</v>
       </c>
       <c r="E10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G10" s="7">
         <v>2</v>
@@ -1837,13 +1831,13 @@
         <v>2</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>9</v>
       </c>
       <c r="E11" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="G11" s="7">
         <v>2</v>
@@ -1863,13 +1857,13 @@
         <v>2</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D12" s="5" t="s">
         <v>9</v>
       </c>
       <c r="E12" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G12" s="7">
         <v>2</v>
@@ -1889,13 +1883,13 @@
         <v>2</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>9</v>
       </c>
       <c r="E13" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="G13" s="7">
         <v>2</v>
@@ -1915,13 +1909,13 @@
         <v>2</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D14" s="8" t="s">
         <v>11</v>
       </c>
       <c r="E14" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="G14" s="7">
         <v>2</v>
@@ -1943,7 +1937,7 @@
       <c r="C15" s="10"/>
       <c r="D15" s="5"/>
       <c r="G15" s="5" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="H15" s="4">
         <f>SUM($G$2:G15)/$G$17</f>
@@ -1956,7 +1950,7 @@
       <c r="C16" s="13"/>
       <c r="D16" s="6"/>
       <c r="E16" s="9" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="G16" s="5">
         <f>SUM(G2:G14)</f>
@@ -1966,7 +1960,7 @@
     </row>
     <row r="17" spans="5:7" x14ac:dyDescent="0.3">
       <c r="E17" s="9" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="G17" s="1">
         <v>24</v>

</xml_diff>

<commit_message>
fix: improve error tracking
</commit_message>
<xml_diff>
--- a/program.xlsx
+++ b/program.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\repos\teaching\AA2627-unibo-mldm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{863F4A4C-8EB3-43A1-A162-8269A9427902}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A24E549-2F7A-4933-ADC4-33D3F940AA06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2304" yWindow="2304" windowWidth="34560" windowHeight="18600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="57480" yWindow="15885" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AA2627" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="57">
   <si>
     <t>When</t>
   </si>
@@ -201,6 +201,12 @@
   </si>
   <si>
     <t>05-NN + Ensemble</t>
+  </si>
+  <si>
+    <t>Lab Clustering</t>
+  </si>
+  <si>
+    <t>(guided lab)</t>
   </si>
 </sst>
 </file>
@@ -974,7 +980,7 @@
       <c r="D14" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E14" s="19" t="s">
         <v>17</v>
       </c>
       <c r="G14" s="7">
@@ -1001,7 +1007,10 @@
         <v>11</v>
       </c>
       <c r="E15" s="15" t="s">
-        <v>19</v>
+        <v>55</v>
+      </c>
+      <c r="F15" t="s">
+        <v>56</v>
       </c>
       <c r="G15" s="7">
         <v>2</v>

</xml_diff>